<commit_message>
fix: changes during testing session
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Repositories/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2317C7-C18E-624B-A375-3D7426836A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CC1FFB-AEAE-224B-8061-0A25F1ECF466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="-28200" windowWidth="34420" windowHeight="28200" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="-28180" windowWidth="34380" windowHeight="28200" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2705" uniqueCount="857">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="863">
   <si>
     <t>Property label</t>
   </si>
@@ -2701,6 +2701,24 @@
   </si>
   <si>
     <t>skos:ConceptScheme (IRI)</t>
+  </si>
+  <si>
+    <t>http://edamontology.org/</t>
+  </si>
+  <si>
+    <t>http://schema.org/</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/prov#</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/oa#</t>
+  </si>
+  <si>
+    <t>^http://snomed\\.info/id/[0-9]{6,18}$</t>
+  </si>
+  <si>
+    <t>^(http://snomed\\.info/id/[0-9]{6,18}|http://id\\.who\\.int/icd/entity/[0-9]+|http://www\\.orpha\\.net/ORDO/Orphanet_[0-9]+)$</t>
   </si>
 </sst>
 </file>
@@ -3715,10 +3733,13 @@
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3731,9 +3752,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7805,7 +7823,7 @@
         <v>75</v>
       </c>
       <c r="P9" s="203" t="s">
-        <v>155</v>
+        <v>76</v>
       </c>
       <c r="S9" s="121" t="b">
         <v>1</v>
@@ -9274,7 +9292,7 @@
         <v>75</v>
       </c>
       <c r="O4" s="27" t="s">
-        <v>155</v>
+        <v>76</v>
       </c>
       <c r="R4" s="27" t="b">
         <v>1</v>
@@ -9354,7 +9372,7 @@
       <c r="I6" s="220" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="219" t="s">
+      <c r="J6" s="213" t="s">
         <v>83</v>
       </c>
       <c r="K6" s="228" t="s">
@@ -9372,13 +9390,13 @@
       <c r="U6" s="91"/>
     </row>
     <row r="7" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="216"/>
-      <c r="B7" s="216"/>
-      <c r="C7" s="216"/>
+      <c r="A7" s="217"/>
+      <c r="B7" s="217"/>
+      <c r="C7" s="217"/>
       <c r="D7" s="179" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="216"/>
+      <c r="E7" s="217"/>
       <c r="F7" s="214"/>
       <c r="G7" s="214"/>
       <c r="H7" s="214"/>
@@ -9388,13 +9406,13 @@
       <c r="L7" s="214"/>
     </row>
     <row r="8" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="216"/>
-      <c r="B8" s="216"/>
-      <c r="C8" s="216"/>
+      <c r="A8" s="217"/>
+      <c r="B8" s="217"/>
+      <c r="C8" s="217"/>
       <c r="D8" s="179" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="216"/>
+      <c r="E8" s="217"/>
       <c r="F8" s="214"/>
       <c r="G8" s="214"/>
       <c r="H8" s="214"/>
@@ -9404,13 +9422,13 @@
       <c r="L8" s="214"/>
     </row>
     <row r="9" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="216"/>
-      <c r="B9" s="216"/>
-      <c r="C9" s="216"/>
+      <c r="A9" s="217"/>
+      <c r="B9" s="217"/>
+      <c r="C9" s="217"/>
       <c r="D9" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="216"/>
+      <c r="E9" s="217"/>
       <c r="F9" s="214"/>
       <c r="G9" s="214"/>
       <c r="H9" s="214"/>
@@ -9420,13 +9438,13 @@
       <c r="L9" s="214"/>
     </row>
     <row r="10" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="216"/>
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
+      <c r="A10" s="217"/>
+      <c r="B10" s="217"/>
+      <c r="C10" s="217"/>
       <c r="D10" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="E10" s="216"/>
+      <c r="E10" s="217"/>
       <c r="F10" s="214"/>
       <c r="G10" s="214"/>
       <c r="H10" s="214"/>
@@ -9802,17 +9820,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
   <mergeCells count="11">
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="E6:E10"/>
+    <mergeCell ref="C6:C10"/>
     <mergeCell ref="I6:I10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="L6:L10"/>
     <mergeCell ref="K6:K10"/>
     <mergeCell ref="F6:F10"/>
     <mergeCell ref="J6:J10"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="E6:E10"/>
-    <mergeCell ref="C6:C10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="226" priority="11" operator="equal">
@@ -10928,6 +10946,9 @@
       <c r="O22" t="s">
         <v>33</v>
       </c>
+      <c r="Q22" s="200" t="s">
+        <v>492</v>
+      </c>
       <c r="S22" s="87"/>
       <c r="T22" s="87"/>
       <c r="U22" s="87"/>
@@ -11554,6 +11575,7 @@
     <hyperlink ref="D16" r:id="rId4" xr:uid="{00000000-0004-0000-0B00-000003000000}"/>
     <hyperlink ref="D17" r:id="rId5" xr:uid="{00000000-0004-0000-0B00-000004000000}"/>
     <hyperlink ref="D22" r:id="rId6" xr:uid="{00000000-0004-0000-0B00-000005000000}"/>
+    <hyperlink ref="Q22" r:id="rId7" tooltip="http://publications.europa.eu/resource/authority/data-theme/heal" xr:uid="{3B9F00E5-3EDE-1A4B-8670-8337B0670862}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12876,6 +12898,9 @@
       </c>
       <c r="Q2" s="2" t="s">
         <v>155</v>
+      </c>
+      <c r="T2" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="U2" s="31"/>
       <c r="V2" s="31"/>
@@ -14396,7 +14421,7 @@
         <v>75</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="U3" s="36"/>
       <c r="V3" s="36"/>
@@ -16195,6 +16220,9 @@
       <c r="Q3" s="27" t="s">
         <v>155</v>
       </c>
+      <c r="T3" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="U3" s="36"/>
       <c r="V3" s="36"/>
       <c r="W3" s="36"/>
@@ -17115,7 +17143,7 @@
         <v>73</v>
       </c>
       <c r="H2" s="168" t="s">
-        <v>67</v>
+        <v>730</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>29</v>
@@ -17170,6 +17198,9 @@
       <c r="Q3" s="27" t="s">
         <v>155</v>
       </c>
+      <c r="T3" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="U3" s="36"/>
       <c r="V3" s="36"/>
       <c r="W3" s="36"/>
@@ -17209,7 +17240,10 @@
         <v>75</v>
       </c>
       <c r="Q4" s="27" t="s">
-        <v>155</v>
+        <v>76</v>
+      </c>
+      <c r="T4" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="U4" s="13"/>
       <c r="V4" s="13"/>
@@ -18176,20 +18210,32 @@
       <c r="A22" t="s">
         <v>198</v>
       </c>
+      <c r="B22" s="200" t="s">
+        <v>857</v>
+      </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>199</v>
       </c>
+      <c r="B23" s="200" t="s">
+        <v>860</v>
+      </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>200</v>
       </c>
+      <c r="B24" s="200" t="s">
+        <v>859</v>
+      </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>201</v>
+      </c>
+      <c r="B25" s="200" t="s">
+        <v>858</v>
       </c>
     </row>
   </sheetData>
@@ -18212,6 +18258,10 @@
     <hyperlink ref="B19" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
     <hyperlink ref="B20" r:id="rId17" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
     <hyperlink ref="B21" r:id="rId18" xr:uid="{00000000-0004-0000-0200-000011000000}"/>
+    <hyperlink ref="B22" r:id="rId19" tooltip="http://edamontology.org/" xr:uid="{58418185-E732-F945-80DB-5E6738BC5BA8}"/>
+    <hyperlink ref="B25" r:id="rId20" tooltip="http://schema.org/" xr:uid="{DEAFF9D5-EB1E-F040-8316-167366B3631C}"/>
+    <hyperlink ref="B24" r:id="rId21" tooltip="http://www.w3.org/ns/prov#" display="http://www.w3.org/ns/prov" xr:uid="{9A1C84E5-E39B-B743-BD5F-D063A07D12B0}"/>
+    <hyperlink ref="B23" r:id="rId22" tooltip="http://www.w3.org/ns/oa#" display="http://www.w3.org/ns/oa" xr:uid="{962971F1-479E-7446-ADCB-7507A33072DE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19002,41 +19052,41 @@
       <c r="V7" s="91"/>
     </row>
     <row r="8" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="217" t="s">
+      <c r="A8" s="218" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="215" t="s">
+      <c r="B8" s="216" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="217" t="s">
+      <c r="C8" s="218" t="s">
         <v>79</v>
       </c>
       <c r="D8" s="176" t="s">
         <v>80</v>
       </c>
-      <c r="E8" s="218" t="s">
+      <c r="E8" s="219" t="s">
         <v>81</v>
       </c>
-      <c r="F8" s="213" t="s">
+      <c r="F8" s="215" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="213" t="s">
+      <c r="G8" s="215" t="s">
         <v>82</v>
       </c>
-      <c r="H8" s="213" t="s">
+      <c r="H8" s="215" t="s">
         <v>28</v>
       </c>
-      <c r="I8" s="219" t="s">
+      <c r="I8" s="213" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="219" t="s">
+      <c r="J8" s="213" t="s">
         <v>83</v>
       </c>
       <c r="K8" s="103"/>
-      <c r="L8" s="219"/>
-      <c r="M8" s="219"/>
+      <c r="L8" s="213"/>
+      <c r="M8" s="213"/>
       <c r="O8" s="27" t="s">
-        <v>32</v>
+        <v>417</v>
       </c>
       <c r="P8" s="27" t="s">
         <v>33</v>
@@ -19047,13 +19097,13 @@
       <c r="V8" s="87"/>
     </row>
     <row r="9" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="216"/>
-      <c r="B9" s="216"/>
-      <c r="C9" s="216"/>
+      <c r="A9" s="217"/>
+      <c r="B9" s="217"/>
+      <c r="C9" s="217"/>
       <c r="D9" s="177" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="216"/>
+      <c r="E9" s="217"/>
       <c r="F9" s="214"/>
       <c r="G9" s="214"/>
       <c r="H9" s="214"/>
@@ -19065,13 +19115,13 @@
       <c r="S9" s="69"/>
     </row>
     <row r="10" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="216"/>
-      <c r="B10" s="216"/>
-      <c r="C10" s="216"/>
+      <c r="A10" s="217"/>
+      <c r="B10" s="217"/>
+      <c r="C10" s="217"/>
       <c r="D10" s="177" t="s">
         <v>85</v>
       </c>
-      <c r="E10" s="216"/>
+      <c r="E10" s="217"/>
       <c r="F10" s="214"/>
       <c r="G10" s="214"/>
       <c r="H10" s="214"/>
@@ -19083,13 +19133,13 @@
       <c r="S10" s="69"/>
     </row>
     <row r="11" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="216"/>
-      <c r="B11" s="216"/>
-      <c r="C11" s="216"/>
+      <c r="A11" s="217"/>
+      <c r="B11" s="217"/>
+      <c r="C11" s="217"/>
       <c r="D11" s="117" t="s">
         <v>86</v>
       </c>
-      <c r="E11" s="216"/>
+      <c r="E11" s="217"/>
       <c r="F11" s="214"/>
       <c r="G11" s="214"/>
       <c r="H11" s="214"/>
@@ -19101,13 +19151,13 @@
       <c r="S11" s="69"/>
     </row>
     <row r="12" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="216"/>
-      <c r="B12" s="216"/>
-      <c r="C12" s="216"/>
+      <c r="A12" s="217"/>
+      <c r="B12" s="217"/>
+      <c r="C12" s="217"/>
       <c r="D12" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="E12" s="216"/>
+      <c r="E12" s="217"/>
       <c r="F12" s="214"/>
       <c r="G12" s="214"/>
       <c r="H12" s="214"/>
@@ -19247,7 +19297,7 @@
       <c r="L15" s="95"/>
       <c r="M15" s="95"/>
       <c r="O15" s="27" t="s">
-        <v>32</v>
+        <v>417</v>
       </c>
       <c r="P15" s="27" t="s">
         <v>33</v>
@@ -19629,7 +19679,7 @@
       <c r="L23" s="95"/>
       <c r="M23" s="95"/>
       <c r="O23" s="27" t="s">
-        <v>32</v>
+        <v>417</v>
       </c>
       <c r="P23" s="27" t="s">
         <v>33</v>
@@ -19691,17 +19741,17 @@
   </sheetData>
   <autoFilter ref="A1:J24" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="11">
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="G8:G12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="J8:J12"/>
     <mergeCell ref="F8:F12"/>
     <mergeCell ref="H8:H12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="C8:C12"/>
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="G8:G12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="309" priority="20" operator="equal">
@@ -20101,6 +20151,9 @@
       <c r="Q5" s="27" t="s">
         <v>33</v>
       </c>
+      <c r="R5" s="27" t="s">
+        <v>861</v>
+      </c>
       <c r="U5" s="91"/>
       <c r="V5" s="91"/>
       <c r="W5" s="91"/>
@@ -20443,7 +20496,7 @@
         <v>75</v>
       </c>
       <c r="Q12" s="27" t="s">
-        <v>155</v>
+        <v>76</v>
       </c>
       <c r="T12" s="27" t="b">
         <v>1</v>
@@ -20657,7 +20710,7 @@
       <c r="E17" s="222" t="s">
         <v>329</v>
       </c>
-      <c r="F17" s="213" t="s">
+      <c r="F17" s="215" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="226" t="s">
@@ -20687,9 +20740,9 @@
       <c r="W17" s="91"/>
     </row>
     <row r="18" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="216"/>
-      <c r="B18" s="216"/>
-      <c r="C18" s="216"/>
+      <c r="A18" s="217"/>
+      <c r="B18" s="217"/>
+      <c r="C18" s="217"/>
       <c r="D18" s="179" t="s">
         <v>84</v>
       </c>
@@ -20705,9 +20758,9 @@
       <c r="N18" s="214"/>
     </row>
     <row r="19" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="216"/>
-      <c r="B19" s="216"/>
-      <c r="C19" s="216"/>
+      <c r="A19" s="217"/>
+      <c r="B19" s="217"/>
+      <c r="C19" s="217"/>
       <c r="D19" s="179" t="s">
         <v>85</v>
       </c>
@@ -20723,9 +20776,9 @@
       <c r="N19" s="214"/>
     </row>
     <row r="20" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="216"/>
-      <c r="B20" s="216"/>
-      <c r="C20" s="216"/>
+      <c r="A20" s="217"/>
+      <c r="B20" s="217"/>
+      <c r="C20" s="217"/>
       <c r="D20" s="105" t="s">
         <v>86</v>
       </c>
@@ -20741,9 +20794,9 @@
       <c r="N20" s="214"/>
     </row>
     <row r="21" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="216"/>
-      <c r="B21" s="216"/>
-      <c r="C21" s="216"/>
+      <c r="A21" s="217"/>
+      <c r="B21" s="217"/>
+      <c r="C21" s="217"/>
       <c r="D21" s="105" t="s">
         <v>87</v>
       </c>
@@ -20845,6 +20898,9 @@
       </c>
       <c r="Q23" s="27" t="s">
         <v>33</v>
+      </c>
+      <c r="R23" s="27" t="s">
+        <v>862</v>
       </c>
       <c r="U23" s="91"/>
       <c r="V23" s="91"/>
@@ -23096,7 +23152,7 @@
         <v>75</v>
       </c>
       <c r="Y4" s="102" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="AC4" s="45"/>
       <c r="AD4" s="45"/>
@@ -23150,7 +23206,7 @@
         <v>75</v>
       </c>
       <c r="Y5" s="102" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="AB5" s="102" t="b">
         <v>1</v>
@@ -24421,7 +24477,7 @@
         <v>75</v>
       </c>
       <c r="T4" s="102" t="s">
-        <v>76</v>
+        <v>155</v>
       </c>
       <c r="X4" s="45"/>
       <c r="Y4" s="45"/>

</xml_diff>

<commit_message>
fix: added title property to tablegroup class
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Repositories/health-ri-metadata/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61CC1FFB-AEAE-224B-8061-0A25F1ECF466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0BE25E-6F18-694D-9DF3-EA1FE8CFF571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="-28180" windowWidth="34380" windowHeight="28200" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="-28200" windowWidth="34380" windowHeight="28200" firstSheet="8" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2722" uniqueCount="865">
   <si>
     <t>Property label</t>
   </si>
@@ -2719,6 +2719,12 @@
   </si>
   <si>
     <t>^(http://snomed\\.info/id/[0-9]{6,18}|http://id\\.who\\.int/icd/entity/[0-9]+|http://www\\.orpha\\.net/ORDO/Orphanet_[0-9]+)$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Table group title.</t>
+  </si>
+  <si>
+    <t>Used to provide a human-readable title for the table group. Can appear in multiple languages.</t>
   </si>
 </sst>
 </file>
@@ -3733,13 +3739,10 @@
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3752,6 +3755,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -9372,7 +9378,7 @@
       <c r="I6" s="220" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="213" t="s">
+      <c r="J6" s="219" t="s">
         <v>83</v>
       </c>
       <c r="K6" s="228" t="s">
@@ -9390,13 +9396,13 @@
       <c r="U6" s="91"/>
     </row>
     <row r="7" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="217"/>
-      <c r="B7" s="217"/>
-      <c r="C7" s="217"/>
+      <c r="A7" s="216"/>
+      <c r="B7" s="216"/>
+      <c r="C7" s="216"/>
       <c r="D7" s="179" t="s">
         <v>84</v>
       </c>
-      <c r="E7" s="217"/>
+      <c r="E7" s="216"/>
       <c r="F7" s="214"/>
       <c r="G7" s="214"/>
       <c r="H7" s="214"/>
@@ -9406,13 +9412,13 @@
       <c r="L7" s="214"/>
     </row>
     <row r="8" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="217"/>
-      <c r="B8" s="217"/>
-      <c r="C8" s="217"/>
+      <c r="A8" s="216"/>
+      <c r="B8" s="216"/>
+      <c r="C8" s="216"/>
       <c r="D8" s="179" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="217"/>
+      <c r="E8" s="216"/>
       <c r="F8" s="214"/>
       <c r="G8" s="214"/>
       <c r="H8" s="214"/>
@@ -9422,13 +9428,13 @@
       <c r="L8" s="214"/>
     </row>
     <row r="9" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="217"/>
-      <c r="B9" s="217"/>
-      <c r="C9" s="217"/>
+      <c r="A9" s="216"/>
+      <c r="B9" s="216"/>
+      <c r="C9" s="216"/>
       <c r="D9" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="217"/>
+      <c r="E9" s="216"/>
       <c r="F9" s="214"/>
       <c r="G9" s="214"/>
       <c r="H9" s="214"/>
@@ -9438,13 +9444,13 @@
       <c r="L9" s="214"/>
     </row>
     <row r="10" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="217"/>
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
+      <c r="A10" s="216"/>
+      <c r="B10" s="216"/>
+      <c r="C10" s="216"/>
       <c r="D10" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="E10" s="217"/>
+      <c r="E10" s="216"/>
       <c r="F10" s="214"/>
       <c r="G10" s="214"/>
       <c r="H10" s="214"/>
@@ -9820,17 +9826,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
   <mergeCells count="11">
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="E6:E10"/>
-    <mergeCell ref="C6:C10"/>
     <mergeCell ref="I6:I10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="L6:L10"/>
     <mergeCell ref="K6:K10"/>
     <mergeCell ref="F6:F10"/>
     <mergeCell ref="J6:J10"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="E6:E10"/>
+    <mergeCell ref="C6:C10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="226" priority="11" operator="equal">
@@ -15308,15 +15314,40 @@
       <c r="V2" s="31"/>
       <c r="W2" s="31"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A3" s="13"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="4"/>
+    <row r="3" spans="1:23" ht="56" x14ac:dyDescent="0.2">
+      <c r="A3" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>863</v>
+      </c>
+      <c r="C3" s="41" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>864</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="T3" s="2" t="b">
+        <v>1</v>
+      </c>
       <c r="U3" s="13"/>
       <c r="V3" s="13"/>
       <c r="W3" s="13"/>
@@ -19052,39 +19083,39 @@
       <c r="V7" s="91"/>
     </row>
     <row r="8" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="218" t="s">
+      <c r="A8" s="217" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="216" t="s">
+      <c r="B8" s="215" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="218" t="s">
+      <c r="C8" s="217" t="s">
         <v>79</v>
       </c>
       <c r="D8" s="176" t="s">
         <v>80</v>
       </c>
-      <c r="E8" s="219" t="s">
+      <c r="E8" s="218" t="s">
         <v>81</v>
       </c>
-      <c r="F8" s="215" t="s">
+      <c r="F8" s="213" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="215" t="s">
+      <c r="G8" s="213" t="s">
         <v>82</v>
       </c>
-      <c r="H8" s="215" t="s">
+      <c r="H8" s="213" t="s">
         <v>28</v>
       </c>
-      <c r="I8" s="213" t="s">
+      <c r="I8" s="219" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="213" t="s">
+      <c r="J8" s="219" t="s">
         <v>83</v>
       </c>
       <c r="K8" s="103"/>
-      <c r="L8" s="213"/>
-      <c r="M8" s="213"/>
+      <c r="L8" s="219"/>
+      <c r="M8" s="219"/>
       <c r="O8" s="27" t="s">
         <v>417</v>
       </c>
@@ -19097,13 +19128,13 @@
       <c r="V8" s="87"/>
     </row>
     <row r="9" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="217"/>
-      <c r="B9" s="217"/>
-      <c r="C9" s="217"/>
+      <c r="A9" s="216"/>
+      <c r="B9" s="216"/>
+      <c r="C9" s="216"/>
       <c r="D9" s="177" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="217"/>
+      <c r="E9" s="216"/>
       <c r="F9" s="214"/>
       <c r="G9" s="214"/>
       <c r="H9" s="214"/>
@@ -19115,13 +19146,13 @@
       <c r="S9" s="69"/>
     </row>
     <row r="10" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="217"/>
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
+      <c r="A10" s="216"/>
+      <c r="B10" s="216"/>
+      <c r="C10" s="216"/>
       <c r="D10" s="177" t="s">
         <v>85</v>
       </c>
-      <c r="E10" s="217"/>
+      <c r="E10" s="216"/>
       <c r="F10" s="214"/>
       <c r="G10" s="214"/>
       <c r="H10" s="214"/>
@@ -19133,13 +19164,13 @@
       <c r="S10" s="69"/>
     </row>
     <row r="11" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="217"/>
-      <c r="B11" s="217"/>
-      <c r="C11" s="217"/>
+      <c r="A11" s="216"/>
+      <c r="B11" s="216"/>
+      <c r="C11" s="216"/>
       <c r="D11" s="117" t="s">
         <v>86</v>
       </c>
-      <c r="E11" s="217"/>
+      <c r="E11" s="216"/>
       <c r="F11" s="214"/>
       <c r="G11" s="214"/>
       <c r="H11" s="214"/>
@@ -19151,13 +19182,13 @@
       <c r="S11" s="69"/>
     </row>
     <row r="12" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="217"/>
-      <c r="B12" s="217"/>
-      <c r="C12" s="217"/>
+      <c r="A12" s="216"/>
+      <c r="B12" s="216"/>
+      <c r="C12" s="216"/>
       <c r="D12" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="E12" s="217"/>
+      <c r="E12" s="216"/>
       <c r="F12" s="214"/>
       <c r="G12" s="214"/>
       <c r="H12" s="214"/>
@@ -19741,17 +19772,17 @@
   </sheetData>
   <autoFilter ref="A1:J24" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="11">
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="G8:G12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="J8:J12"/>
     <mergeCell ref="F8:F12"/>
     <mergeCell ref="H8:H12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="C8:C12"/>
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="G8:G12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="309" priority="20" operator="equal">
@@ -20710,7 +20741,7 @@
       <c r="E17" s="222" t="s">
         <v>329</v>
       </c>
-      <c r="F17" s="215" t="s">
+      <c r="F17" s="213" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="226" t="s">
@@ -20740,9 +20771,9 @@
       <c r="W17" s="91"/>
     </row>
     <row r="18" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="217"/>
-      <c r="B18" s="217"/>
-      <c r="C18" s="217"/>
+      <c r="A18" s="216"/>
+      <c r="B18" s="216"/>
+      <c r="C18" s="216"/>
       <c r="D18" s="179" t="s">
         <v>84</v>
       </c>
@@ -20758,9 +20789,9 @@
       <c r="N18" s="214"/>
     </row>
     <row r="19" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="217"/>
-      <c r="B19" s="217"/>
-      <c r="C19" s="217"/>
+      <c r="A19" s="216"/>
+      <c r="B19" s="216"/>
+      <c r="C19" s="216"/>
       <c r="D19" s="179" t="s">
         <v>85</v>
       </c>
@@ -20776,9 +20807,9 @@
       <c r="N19" s="214"/>
     </row>
     <row r="20" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="217"/>
-      <c r="B20" s="217"/>
-      <c r="C20" s="217"/>
+      <c r="A20" s="216"/>
+      <c r="B20" s="216"/>
+      <c r="C20" s="216"/>
       <c r="D20" s="105" t="s">
         <v>86</v>
       </c>
@@ -20794,9 +20825,9 @@
       <c r="N20" s="214"/>
     </row>
     <row r="21" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="217"/>
-      <c r="B21" s="217"/>
-      <c r="C21" s="217"/>
+      <c r="A21" s="216"/>
+      <c r="B21" s="216"/>
+      <c r="C21" s="216"/>
       <c r="D21" s="105" t="s">
         <v>87</v>
       </c>

</xml_diff>

<commit_message>
feat: added SHACL information for TableGroup dct:title
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Repositories/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0BE25E-6F18-694D-9DF3-EA1FE8CFF571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF62ED4D-409F-E34E-ADE3-AC8BCFFF45B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="-28200" windowWidth="34380" windowHeight="28200" firstSheet="8" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="-28200" windowWidth="34380" windowHeight="28200" firstSheet="8" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2722" uniqueCount="865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="865">
   <si>
     <t>Property label</t>
   </si>
@@ -15345,6 +15345,12 @@
       <c r="J3" s="2" t="s">
         <v>83</v>
       </c>
+      <c r="P3" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q3" s="27" t="s">
+        <v>155</v>
+      </c>
       <c r="T3" s="2" t="b">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
feat: adds Data Service as resources in FDP
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Repositories/temp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderharms/Documents/Repositories/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CDC95C-5D4F-794F-9990-F0E4C0D999D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFAA4EFD-C56C-4E4B-A331-3A5335396BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="20540" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="780" windowWidth="36000" windowHeight="20540" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2746" uniqueCount="879">
   <si>
     <t>Property label</t>
   </si>
@@ -2764,6 +2764,9 @@
   </si>
   <si>
     <t>Sample Distribution</t>
+  </si>
+  <si>
+    <t>Data Service</t>
   </si>
 </sst>
 </file>
@@ -3808,32 +3811,17 @@
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -3844,6 +3832,9 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3851,6 +3842,18 @@
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -3865,7 +3868,47 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="322">
+  <dxfs count="326">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -7431,7 +7474,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:V58"/>
+  <dimension ref="A1:W58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" style="9" customWidth="1"/>
@@ -7448,12 +7491,12 @@
     <col min="12" max="12" width="28.1640625" style="2" customWidth="1"/>
     <col min="13" max="13" width="28.83203125" style="2" customWidth="1"/>
     <col min="14" max="14" width="9.1640625" style="2" customWidth="1"/>
-    <col min="15" max="19" width="9.1640625" style="2"/>
-    <col min="20" max="22" width="19.1640625" customWidth="1"/>
-    <col min="23" max="16384" width="9.1640625" style="2"/>
+    <col min="15" max="20" width="9.1640625" style="2"/>
+    <col min="21" max="23" width="19.1640625" customWidth="1"/>
+    <col min="24" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="165" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" s="165" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
@@ -7511,17 +7554,20 @@
       <c r="S1" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="63" t="s">
+      <c r="T1" s="66" t="s">
+        <v>874</v>
+      </c>
+      <c r="U1" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="63" t="s">
+      <c r="V1" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="63" t="s">
+      <c r="W1" s="63" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="91" t="s">
         <v>624</v>
       </c>
@@ -7571,11 +7617,14 @@
         <v>195</v>
       </c>
       <c r="S2" s="121"/>
-      <c r="T2" s="91"/>
+      <c r="T2" s="2" t="s">
+        <v>878</v>
+      </c>
       <c r="U2" s="91"/>
       <c r="V2" s="91"/>
-    </row>
-    <row r="3" spans="1:22" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W2" s="91"/>
+    </row>
+    <row r="3" spans="1:23" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="87" t="s">
         <v>630</v>
       </c>
@@ -7618,11 +7667,11 @@
         <v>57</v>
       </c>
       <c r="S3" s="121"/>
-      <c r="T3" s="87"/>
       <c r="U3" s="87"/>
       <c r="V3" s="87"/>
-    </row>
-    <row r="4" spans="1:22" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W3" s="87"/>
+    </row>
+    <row r="4" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="91" t="s">
         <v>179</v>
       </c>
@@ -7665,11 +7714,11 @@
         <v>57</v>
       </c>
       <c r="S4" s="121"/>
-      <c r="T4" s="91"/>
       <c r="U4" s="91"/>
       <c r="V4" s="91"/>
-    </row>
-    <row r="5" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W4" s="91"/>
+    </row>
+    <row r="5" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="97" t="s">
         <v>636</v>
       </c>
@@ -7710,11 +7759,11 @@
         <v>57</v>
       </c>
       <c r="S5" s="121"/>
-      <c r="T5" s="97"/>
       <c r="U5" s="97"/>
       <c r="V5" s="97"/>
-    </row>
-    <row r="6" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W5" s="97"/>
+    </row>
+    <row r="6" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="91" t="s">
         <v>641</v>
       </c>
@@ -7757,11 +7806,11 @@
         <v>34</v>
       </c>
       <c r="S6" s="121"/>
-      <c r="T6" s="91"/>
       <c r="U6" s="91"/>
       <c r="V6" s="91"/>
-    </row>
-    <row r="7" spans="1:22" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W6" s="91"/>
+    </row>
+    <row r="7" spans="1:23" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="87" t="s">
         <v>646</v>
       </c>
@@ -7811,11 +7860,11 @@
         <v>195</v>
       </c>
       <c r="S7" s="121"/>
-      <c r="T7" s="87"/>
       <c r="U7" s="87"/>
       <c r="V7" s="87"/>
-    </row>
-    <row r="8" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W7" s="87"/>
+    </row>
+    <row r="8" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="91" t="s">
         <v>653</v>
       </c>
@@ -7858,11 +7907,11 @@
         <v>57</v>
       </c>
       <c r="S8" s="121"/>
-      <c r="T8" s="91"/>
       <c r="U8" s="91"/>
       <c r="V8" s="91"/>
-    </row>
-    <row r="9" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W8" s="91"/>
+    </row>
+    <row r="9" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="87" t="s">
         <v>40</v>
       </c>
@@ -7907,11 +7956,11 @@
       <c r="S9" s="121" t="b">
         <v>1</v>
       </c>
-      <c r="T9" s="87"/>
       <c r="U9" s="87"/>
       <c r="V9" s="87"/>
-    </row>
-    <row r="10" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W9" s="87"/>
+    </row>
+    <row r="10" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="91" t="s">
         <v>350</v>
       </c>
@@ -7954,11 +8003,11 @@
         <v>57</v>
       </c>
       <c r="S10" s="121"/>
-      <c r="T10" s="91"/>
       <c r="U10" s="91"/>
       <c r="V10" s="91"/>
-    </row>
-    <row r="11" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W10" s="91"/>
+    </row>
+    <row r="11" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="87" t="s">
         <v>664</v>
       </c>
@@ -8001,11 +8050,11 @@
         <v>57</v>
       </c>
       <c r="S11" s="121"/>
-      <c r="T11" s="87"/>
       <c r="U11" s="87"/>
       <c r="V11" s="87"/>
-    </row>
-    <row r="12" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W11" s="87"/>
+    </row>
+    <row r="12" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="91" t="s">
         <v>669</v>
       </c>
@@ -8048,11 +8097,11 @@
         <v>57</v>
       </c>
       <c r="S12" s="121"/>
-      <c r="T12" s="91"/>
       <c r="U12" s="91"/>
       <c r="V12" s="91"/>
-    </row>
-    <row r="13" spans="1:22" ht="99" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W12" s="91"/>
+    </row>
+    <row r="13" spans="1:23" ht="99" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="87" t="s">
         <v>241</v>
       </c>
@@ -8095,11 +8144,11 @@
         <v>57</v>
       </c>
       <c r="S13" s="121"/>
-      <c r="T13" s="87"/>
       <c r="U13" s="87"/>
       <c r="V13" s="87"/>
-    </row>
-    <row r="14" spans="1:22" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W13" s="87"/>
+    </row>
+    <row r="14" spans="1:23" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="91" t="s">
         <v>248</v>
       </c>
@@ -8142,11 +8191,11 @@
         <v>57</v>
       </c>
       <c r="S14" s="121"/>
-      <c r="T14" s="91"/>
       <c r="U14" s="91"/>
       <c r="V14" s="91"/>
-    </row>
-    <row r="15" spans="1:22" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W14" s="91"/>
+    </row>
+    <row r="15" spans="1:23" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="87" t="s">
         <v>680</v>
       </c>
@@ -8189,11 +8238,11 @@
         <v>57</v>
       </c>
       <c r="S15" s="121"/>
-      <c r="T15" s="87"/>
       <c r="U15" s="87"/>
       <c r="V15" s="87"/>
-    </row>
-    <row r="16" spans="1:22" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W15" s="87"/>
+    </row>
+    <row r="16" spans="1:23" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="91" t="s">
         <v>683</v>
       </c>
@@ -8236,11 +8285,11 @@
         <v>57</v>
       </c>
       <c r="S16" s="121"/>
-      <c r="T16" s="91"/>
       <c r="U16" s="91"/>
       <c r="V16" s="91"/>
-    </row>
-    <row r="17" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W16" s="91"/>
+    </row>
+    <row r="17" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="87" t="s">
         <v>255</v>
       </c>
@@ -8285,11 +8334,11 @@
         <v>261</v>
       </c>
       <c r="S17" s="69"/>
-      <c r="T17" s="87"/>
       <c r="U17" s="87"/>
       <c r="V17" s="87"/>
-    </row>
-    <row r="18" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W17" s="87"/>
+    </row>
+    <row r="18" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="91" t="s">
         <v>689</v>
       </c>
@@ -8332,11 +8381,11 @@
         <v>57</v>
       </c>
       <c r="S18" s="121"/>
-      <c r="T18" s="91"/>
       <c r="U18" s="91"/>
       <c r="V18" s="91"/>
-    </row>
-    <row r="19" spans="1:22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W18" s="91"/>
+    </row>
+    <row r="19" spans="1:23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="87" t="s">
         <v>268</v>
       </c>
@@ -8383,11 +8432,11 @@
         <v>261</v>
       </c>
       <c r="S19" s="69"/>
-      <c r="T19" s="87"/>
       <c r="U19" s="87"/>
       <c r="V19" s="87"/>
-    </row>
-    <row r="20" spans="1:22" ht="231" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W19" s="87"/>
+    </row>
+    <row r="20" spans="1:23" ht="231" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="91" t="s">
         <v>494</v>
       </c>
@@ -8433,11 +8482,11 @@
         <v>195</v>
       </c>
       <c r="S20" s="121"/>
-      <c r="T20" s="91"/>
       <c r="U20" s="91"/>
       <c r="V20" s="91"/>
-    </row>
-    <row r="21" spans="1:22" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W20" s="91"/>
+    </row>
+    <row r="21" spans="1:23" ht="112" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="87" t="s">
         <v>272</v>
       </c>
@@ -8480,11 +8529,11 @@
         <v>57</v>
       </c>
       <c r="S21" s="121"/>
-      <c r="T21" s="87"/>
       <c r="U21" s="87"/>
       <c r="V21" s="87"/>
-    </row>
-    <row r="22" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W21" s="87"/>
+    </row>
+    <row r="22" spans="1:23" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="91" t="s">
         <v>512</v>
       </c>
@@ -8527,11 +8576,11 @@
         <v>57</v>
       </c>
       <c r="S22" s="121"/>
-      <c r="T22" s="91"/>
       <c r="U22" s="91"/>
       <c r="V22" s="91"/>
-    </row>
-    <row r="23" spans="1:22" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W22" s="91"/>
+    </row>
+    <row r="23" spans="1:23" ht="64" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="87" t="s">
         <v>519</v>
       </c>
@@ -8572,11 +8621,11 @@
         <v>34</v>
       </c>
       <c r="S23" s="121"/>
-      <c r="T23" s="87"/>
       <c r="U23" s="87"/>
       <c r="V23" s="87"/>
-    </row>
-    <row r="24" spans="1:22" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W23" s="87"/>
+    </row>
+    <row r="24" spans="1:23" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="91" t="s">
         <v>35</v>
       </c>
@@ -8621,11 +8670,11 @@
       <c r="S24" s="121" t="b">
         <v>1</v>
       </c>
-      <c r="T24" s="91"/>
       <c r="U24" s="91"/>
       <c r="V24" s="91"/>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W24" s="91"/>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" s="21"/>
       <c r="B25" s="8"/>
       <c r="C25" s="21"/>
@@ -8637,11 +8686,11 @@
       <c r="K25" s="70"/>
       <c r="L25" s="27"/>
       <c r="M25" s="27"/>
-      <c r="T25" s="21"/>
       <c r="U25" s="21"/>
       <c r="V25" s="21"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W25" s="21"/>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" s="21"/>
       <c r="B26" s="8"/>
       <c r="C26" s="26"/>
@@ -8653,11 +8702,11 @@
       <c r="K26" s="68"/>
       <c r="L26" s="27"/>
       <c r="M26" s="27"/>
-      <c r="T26" s="21"/>
       <c r="U26" s="21"/>
       <c r="V26" s="21"/>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W26" s="21"/>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" s="21"/>
       <c r="B27" s="8"/>
       <c r="C27" s="21"/>
@@ -8667,11 +8716,11 @@
       <c r="G27" s="20"/>
       <c r="H27" s="22"/>
       <c r="K27" s="70"/>
-      <c r="T27" s="21"/>
       <c r="U27" s="21"/>
       <c r="V27" s="21"/>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W27" s="21"/>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="21"/>
       <c r="B28" s="8"/>
       <c r="D28" s="23"/>
@@ -8680,11 +8729,11 @@
       <c r="G28" s="20"/>
       <c r="H28" s="22"/>
       <c r="K28" s="68"/>
-      <c r="T28" s="21"/>
       <c r="U28" s="21"/>
       <c r="V28" s="21"/>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W28" s="21"/>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" s="21"/>
       <c r="B29" s="8"/>
       <c r="C29" s="21"/>
@@ -8694,11 +8743,11 @@
       <c r="G29" s="20"/>
       <c r="H29" s="22"/>
       <c r="K29" s="68"/>
-      <c r="T29" s="21"/>
       <c r="U29" s="21"/>
       <c r="V29" s="21"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W29" s="21"/>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" s="21"/>
       <c r="B30" s="8"/>
       <c r="C30" s="21"/>
@@ -8707,11 +8756,11 @@
       <c r="G30" s="20"/>
       <c r="H30" s="22"/>
       <c r="K30" s="68"/>
-      <c r="T30" s="21"/>
       <c r="U30" s="21"/>
       <c r="V30" s="21"/>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W30" s="21"/>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="21"/>
       <c r="B31" s="8"/>
       <c r="C31" s="21"/>
@@ -8721,11 +8770,11 @@
       <c r="G31" s="20"/>
       <c r="H31" s="22"/>
       <c r="K31" s="68"/>
-      <c r="T31" s="21"/>
       <c r="U31" s="21"/>
       <c r="V31" s="21"/>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W31" s="21"/>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
       <c r="B32" s="8"/>
       <c r="C32" s="26"/>
@@ -8735,11 +8784,11 @@
       <c r="G32" s="20"/>
       <c r="H32" s="22"/>
       <c r="K32" s="68"/>
-      <c r="T32" s="21"/>
       <c r="U32" s="21"/>
       <c r="V32" s="21"/>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W32" s="21"/>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
       <c r="B33" s="8"/>
       <c r="C33" s="21"/>
@@ -8749,11 +8798,11 @@
       <c r="G33" s="20"/>
       <c r="H33" s="22"/>
       <c r="K33" s="68"/>
-      <c r="T33" s="21"/>
       <c r="U33" s="21"/>
       <c r="V33" s="21"/>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W33" s="21"/>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
       <c r="B34" s="8"/>
       <c r="D34" s="23"/>
@@ -8762,11 +8811,11 @@
       <c r="G34" s="20"/>
       <c r="H34" s="22"/>
       <c r="K34" s="72"/>
-      <c r="T34" s="21"/>
       <c r="U34" s="21"/>
       <c r="V34" s="21"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W34" s="21"/>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="8"/>
       <c r="C35" s="21"/>
@@ -8776,11 +8825,11 @@
       <c r="G35" s="20"/>
       <c r="H35" s="22"/>
       <c r="K35" s="68"/>
-      <c r="T35" s="21"/>
       <c r="U35" s="21"/>
       <c r="V35" s="21"/>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W35" s="21"/>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
       <c r="B36" s="8"/>
       <c r="C36" s="21"/>
@@ -8789,11 +8838,11 @@
       <c r="G36" s="20"/>
       <c r="H36" s="22"/>
       <c r="K36" s="68"/>
-      <c r="T36" s="21"/>
       <c r="U36" s="21"/>
       <c r="V36" s="21"/>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W36" s="21"/>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
       <c r="B37" s="8"/>
       <c r="C37" s="21"/>
@@ -8803,11 +8852,11 @@
       <c r="G37" s="20"/>
       <c r="H37" s="22"/>
       <c r="K37" s="68"/>
-      <c r="T37" s="21"/>
       <c r="U37" s="21"/>
       <c r="V37" s="21"/>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W37" s="21"/>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="8"/>
       <c r="C38" s="26"/>
@@ -8817,11 +8866,11 @@
       <c r="G38" s="20"/>
       <c r="H38" s="22"/>
       <c r="K38" s="68"/>
-      <c r="T38" s="21"/>
       <c r="U38" s="21"/>
       <c r="V38" s="21"/>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W38" s="21"/>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
       <c r="B39" s="8"/>
       <c r="C39" s="21"/>
@@ -8831,11 +8880,11 @@
       <c r="G39" s="20"/>
       <c r="H39" s="22"/>
       <c r="K39" s="68"/>
-      <c r="T39" s="21"/>
       <c r="U39" s="21"/>
       <c r="V39" s="21"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W39" s="21"/>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="21"/>
       <c r="B40" s="8"/>
       <c r="C40" s="21"/>
@@ -8844,11 +8893,11 @@
       <c r="G40" s="20"/>
       <c r="H40" s="22"/>
       <c r="K40" s="68"/>
-      <c r="T40" s="21"/>
       <c r="U40" s="21"/>
       <c r="V40" s="21"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W40" s="21"/>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="21"/>
       <c r="B41" s="8"/>
       <c r="C41" s="21"/>
@@ -8858,11 +8907,11 @@
       <c r="G41" s="20"/>
       <c r="H41" s="22"/>
       <c r="K41" s="68"/>
-      <c r="T41" s="21"/>
       <c r="U41" s="21"/>
       <c r="V41" s="21"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W41" s="21"/>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" s="21"/>
       <c r="B42" s="8"/>
       <c r="C42" s="26"/>
@@ -8872,11 +8921,11 @@
       <c r="G42" s="20"/>
       <c r="H42" s="22"/>
       <c r="K42" s="68"/>
-      <c r="T42" s="21"/>
       <c r="U42" s="21"/>
       <c r="V42" s="21"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W42" s="21"/>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" s="21"/>
       <c r="B43" s="8"/>
       <c r="C43" s="21"/>
@@ -8886,11 +8935,11 @@
       <c r="G43" s="20"/>
       <c r="H43" s="22"/>
       <c r="K43" s="68"/>
-      <c r="T43" s="21"/>
       <c r="U43" s="21"/>
       <c r="V43" s="21"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W43" s="21"/>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" s="21"/>
       <c r="B44" s="8"/>
       <c r="D44" s="23"/>
@@ -8899,11 +8948,11 @@
       <c r="G44" s="20"/>
       <c r="H44" s="22"/>
       <c r="K44" s="68"/>
-      <c r="T44" s="21"/>
       <c r="U44" s="21"/>
       <c r="V44" s="21"/>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W44" s="21"/>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" s="21"/>
       <c r="B45" s="8"/>
       <c r="C45" s="21"/>
@@ -8913,11 +8962,11 @@
       <c r="G45" s="20"/>
       <c r="H45" s="22"/>
       <c r="K45" s="68"/>
-      <c r="T45" s="21"/>
       <c r="U45" s="21"/>
       <c r="V45" s="21"/>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W45" s="21"/>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" s="21"/>
       <c r="B46" s="8"/>
       <c r="C46" s="21"/>
@@ -8926,11 +8975,11 @@
       <c r="G46" s="20"/>
       <c r="H46" s="22"/>
       <c r="K46" s="68"/>
-      <c r="T46" s="21"/>
       <c r="U46" s="21"/>
       <c r="V46" s="21"/>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W46" s="21"/>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" s="21"/>
       <c r="B47" s="8"/>
       <c r="C47" s="21"/>
@@ -8940,11 +8989,11 @@
       <c r="G47" s="20"/>
       <c r="H47" s="22"/>
       <c r="K47" s="68"/>
-      <c r="T47" s="21"/>
       <c r="U47" s="21"/>
       <c r="V47" s="21"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W47" s="21"/>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" s="21"/>
       <c r="B48" s="8"/>
       <c r="C48" s="26"/>
@@ -8954,11 +9003,11 @@
       <c r="G48" s="20"/>
       <c r="H48" s="22"/>
       <c r="K48" s="68"/>
-      <c r="T48" s="21"/>
       <c r="U48" s="21"/>
       <c r="V48" s="21"/>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W48" s="21"/>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" s="21"/>
       <c r="B49" s="8"/>
       <c r="C49" s="21"/>
@@ -8967,11 +9016,11 @@
       <c r="G49" s="20"/>
       <c r="H49" s="22"/>
       <c r="K49" s="68"/>
-      <c r="T49" s="21"/>
       <c r="U49" s="21"/>
       <c r="V49" s="21"/>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W49" s="21"/>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" s="21"/>
       <c r="B50" s="8"/>
       <c r="C50" s="21"/>
@@ -8980,11 +9029,11 @@
       <c r="G50" s="20"/>
       <c r="H50" s="22"/>
       <c r="K50" s="68"/>
-      <c r="T50" s="21"/>
       <c r="U50" s="21"/>
       <c r="V50" s="21"/>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W50" s="21"/>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" s="21"/>
       <c r="B51" s="8"/>
       <c r="C51" s="21"/>
@@ -8994,11 +9043,11 @@
       <c r="G51" s="20"/>
       <c r="H51" s="22"/>
       <c r="K51" s="68"/>
-      <c r="T51" s="21"/>
       <c r="U51" s="21"/>
       <c r="V51" s="21"/>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W51" s="21"/>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" s="21"/>
       <c r="B52" s="8"/>
       <c r="D52" s="23"/>
@@ -9007,11 +9056,11 @@
       <c r="G52" s="20"/>
       <c r="H52" s="22"/>
       <c r="K52" s="68"/>
-      <c r="T52" s="21"/>
       <c r="U52" s="21"/>
       <c r="V52" s="21"/>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W52" s="21"/>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" s="21"/>
       <c r="B53" s="8"/>
       <c r="C53" s="21"/>
@@ -9021,11 +9070,11 @@
       <c r="G53" s="20"/>
       <c r="H53" s="22"/>
       <c r="K53" s="68"/>
-      <c r="T53" s="21"/>
       <c r="U53" s="21"/>
       <c r="V53" s="21"/>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W53" s="21"/>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" s="21"/>
       <c r="B54" s="8"/>
       <c r="C54" s="21"/>
@@ -9035,73 +9084,87 @@
       <c r="G54" s="20"/>
       <c r="H54" s="22"/>
       <c r="K54" s="68"/>
-      <c r="T54" s="21"/>
       <c r="U54" s="21"/>
       <c r="V54" s="21"/>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W54" s="21"/>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K55" s="68"/>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K56" s="68"/>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K57" s="68"/>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K58" s="69"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J24" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <conditionalFormatting sqref="F2:F54">
-    <cfRule type="cellIs" dxfId="240" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="244" priority="20" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H54">
-    <cfRule type="cellIs" dxfId="239" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="243" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="238" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="242" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F54">
-    <cfRule type="cellIs" dxfId="237" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="241" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="236" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="240" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="235" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="239" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="234" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="238" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J54">
-    <cfRule type="containsText" dxfId="233" priority="13" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="237" priority="17" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="232" priority="14" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="236" priority="18" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="231" priority="15" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="235" priority="19" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:S1">
-    <cfRule type="cellIs" dxfId="230" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="234" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="229" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="233" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="228" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="232" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="227" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="231" priority="8" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T1">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"Optional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9424,40 +9487,40 @@
       <c r="U5" s="87"/>
     </row>
     <row r="6" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="226" t="s">
+      <c r="A6" s="220" t="s">
         <v>221</v>
       </c>
-      <c r="B6" s="230" t="s">
+      <c r="B6" s="226" t="s">
         <v>222</v>
       </c>
-      <c r="C6" s="226" t="s">
+      <c r="C6" s="220" t="s">
         <v>223</v>
       </c>
       <c r="D6" s="178" t="s">
         <v>224</v>
       </c>
-      <c r="E6" s="227" t="s">
+      <c r="E6" s="222" t="s">
         <v>365</v>
       </c>
-      <c r="F6" s="231" t="s">
+      <c r="F6" s="227" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="231" t="s">
+      <c r="G6" s="227" t="s">
         <v>226</v>
       </c>
-      <c r="H6" s="231" t="s">
+      <c r="H6" s="227" t="s">
         <v>183</v>
       </c>
-      <c r="I6" s="225" t="s">
+      <c r="I6" s="218" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="222" t="s">
+      <c r="J6" s="232" t="s">
         <v>32</v>
       </c>
       <c r="K6" s="233" t="s">
         <v>713</v>
       </c>
-      <c r="L6" s="225"/>
+      <c r="L6" s="218"/>
       <c r="N6" s="69" t="s">
         <v>321</v>
       </c>
@@ -9469,68 +9532,68 @@
       <c r="U6" s="91"/>
     </row>
     <row r="7" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="219"/>
-      <c r="B7" s="219"/>
-      <c r="C7" s="219"/>
+      <c r="A7" s="221"/>
+      <c r="B7" s="221"/>
+      <c r="C7" s="221"/>
       <c r="D7" s="179" t="s">
         <v>227</v>
       </c>
-      <c r="E7" s="219"/>
-      <c r="F7" s="223"/>
-      <c r="G7" s="223"/>
-      <c r="H7" s="223"/>
-      <c r="I7" s="223"/>
-      <c r="J7" s="223"/>
+      <c r="E7" s="221"/>
+      <c r="F7" s="219"/>
+      <c r="G7" s="219"/>
+      <c r="H7" s="219"/>
+      <c r="I7" s="219"/>
+      <c r="J7" s="219"/>
       <c r="K7" s="234"/>
-      <c r="L7" s="223"/>
+      <c r="L7" s="219"/>
     </row>
     <row r="8" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="219"/>
-      <c r="B8" s="219"/>
-      <c r="C8" s="219"/>
+      <c r="A8" s="221"/>
+      <c r="B8" s="221"/>
+      <c r="C8" s="221"/>
       <c r="D8" s="179" t="s">
         <v>228</v>
       </c>
-      <c r="E8" s="219"/>
-      <c r="F8" s="223"/>
-      <c r="G8" s="223"/>
-      <c r="H8" s="223"/>
-      <c r="I8" s="223"/>
-      <c r="J8" s="223"/>
+      <c r="E8" s="221"/>
+      <c r="F8" s="219"/>
+      <c r="G8" s="219"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="219"/>
+      <c r="J8" s="219"/>
       <c r="K8" s="234"/>
-      <c r="L8" s="223"/>
+      <c r="L8" s="219"/>
     </row>
     <row r="9" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="219"/>
-      <c r="B9" s="219"/>
-      <c r="C9" s="219"/>
+      <c r="A9" s="221"/>
+      <c r="B9" s="221"/>
+      <c r="C9" s="221"/>
       <c r="D9" s="105" t="s">
         <v>229</v>
       </c>
-      <c r="E9" s="219"/>
-      <c r="F9" s="223"/>
-      <c r="G9" s="223"/>
-      <c r="H9" s="223"/>
-      <c r="I9" s="223"/>
-      <c r="J9" s="223"/>
+      <c r="E9" s="221"/>
+      <c r="F9" s="219"/>
+      <c r="G9" s="219"/>
+      <c r="H9" s="219"/>
+      <c r="I9" s="219"/>
+      <c r="J9" s="219"/>
       <c r="K9" s="234"/>
-      <c r="L9" s="223"/>
+      <c r="L9" s="219"/>
     </row>
     <row r="10" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="219"/>
-      <c r="B10" s="219"/>
-      <c r="C10" s="219"/>
+      <c r="A10" s="221"/>
+      <c r="B10" s="221"/>
+      <c r="C10" s="221"/>
       <c r="D10" s="105" t="s">
         <v>230</v>
       </c>
-      <c r="E10" s="219"/>
-      <c r="F10" s="223"/>
-      <c r="G10" s="223"/>
-      <c r="H10" s="223"/>
-      <c r="I10" s="223"/>
-      <c r="J10" s="223"/>
+      <c r="E10" s="221"/>
+      <c r="F10" s="219"/>
+      <c r="G10" s="219"/>
+      <c r="H10" s="219"/>
+      <c r="I10" s="219"/>
+      <c r="J10" s="219"/>
       <c r="K10" s="234"/>
-      <c r="L10" s="223"/>
+      <c r="L10" s="219"/>
     </row>
     <row r="11" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="87" t="s">
@@ -9912,65 +9975,65 @@
     <mergeCell ref="G6:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="226" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="230" priority="11" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H6 H11 G12:I12">
-    <cfRule type="cellIs" dxfId="225" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="229" priority="12" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="224" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="228" priority="13" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="223" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="227" priority="14" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="222" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="226" priority="15" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="221" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="225" priority="16" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="220" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="224" priority="17" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J6">
-    <cfRule type="containsText" dxfId="219" priority="5" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="223" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="218" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="222" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="217" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="221" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:J15">
-    <cfRule type="containsText" dxfId="216" priority="8" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="220" priority="8" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="215" priority="9" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="219" priority="9" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="214" priority="10" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="218" priority="10" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:R1">
-    <cfRule type="cellIs" dxfId="213" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="217" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="212" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="216" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="211" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="215" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="210" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="214" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11578,54 +11641,54 @@
   </sheetData>
   <autoFilter ref="A1:J23" xr:uid="{00000000-0009-0000-0000-00000B000000}"/>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="209" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="213" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="208" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="212" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="211" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="206" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="210" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="209" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="208" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="203" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="202" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="206" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="201" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="205" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="200" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="204" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:R1">
-    <cfRule type="cellIs" dxfId="199" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="203" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="202" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="197" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="201" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="200" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11844,49 +11907,49 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="195" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="199" priority="9" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="194" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="198" priority="10" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="197" priority="11" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="196" priority="12" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="191" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="195" priority="13" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="190" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="194" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="193" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="192" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="191" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P1:U1">
-    <cfRule type="cellIs" dxfId="186" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="190" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="185" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="188" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="187" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12746,85 +12809,85 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A41:B42">
-    <cfRule type="cellIs" dxfId="182" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="186" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="185" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="184" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="179" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="178" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="181" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="176" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="179" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="174" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="9" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="173" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="10" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="11" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="12" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="170" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="13" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="169" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="173" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="167" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="164" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:X1">
-    <cfRule type="cellIs" dxfId="163" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="166" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="161" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13262,88 +13325,88 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D11:E13">
-    <cfRule type="cellIs" dxfId="159" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="163" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="158" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" dxfId="155" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="157" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F23 A12:B13">
-    <cfRule type="cellIs" dxfId="150" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="154" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="149" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="148" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="152" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F23">
-    <cfRule type="cellIs" dxfId="146" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2">
-    <cfRule type="cellIs" dxfId="145" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="148" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="146" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12 H21:H23">
-    <cfRule type="cellIs" dxfId="141" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="145" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="144" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="139" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="142" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="141" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13568,35 +13631,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="135" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="139" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="134" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="136" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="135" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="130" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="133" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="132" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13799,35 +13862,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="126" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="130" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="125" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="129" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="121" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="123" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14030,35 +14093,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="117" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="116" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="120" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="118" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="112" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="115" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="114" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14253,49 +14316,49 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:E3">
-    <cfRule type="cellIs" dxfId="108" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="104" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="13" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="103" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="14" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="15" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="16" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="17" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="99" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15140,88 +15203,88 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A41:B42">
-    <cfRule type="cellIs" dxfId="95" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="21" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="22" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="23" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="24" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="91" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="25" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="26" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="27" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="28" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
-    <cfRule type="cellIs" dxfId="87" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="82" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G3">
-    <cfRule type="cellIs" dxfId="81" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="16" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="17" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="18" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="19" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="77" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="81" priority="29" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="30" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="75" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16049,90 +16112,90 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D39:E41">
-    <cfRule type="cellIs" dxfId="71" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" dxfId="67" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:F2">
-    <cfRule type="cellIs" dxfId="63" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F2 F4:F51 A40:B41">
-    <cfRule type="cellIs" dxfId="62" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F51">
-    <cfRule type="cellIs" dxfId="58" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2">
-    <cfRule type="cellIs" dxfId="57" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H8 H10:H14 H16:H24 H26:H40 H49:H51">
-    <cfRule type="cellIs" dxfId="53" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="57" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17029,88 +17092,88 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="47" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
-    <cfRule type="cellIs" dxfId="43" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F52 A41:B42">
-    <cfRule type="cellIs" dxfId="38" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="34" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="33" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="29" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18035,88 +18098,88 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="23" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
-    <cfRule type="cellIs" dxfId="19" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F52 A41:B42">
-    <cfRule type="cellIs" dxfId="14" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="10" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="9" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="5" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18766,44 +18829,44 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1 H1:I1">
-    <cfRule type="cellIs" dxfId="321" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="325" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="320" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="324" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="319" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="323" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="318" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="322" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="317" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="321" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="316" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="320" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="315" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="319" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="314" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="318" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:Q1">
-    <cfRule type="cellIs" dxfId="313" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="317" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="312" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="316" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="311" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="315" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="310" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="314" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19213,39 +19276,39 @@
       <c r="V7" s="91"/>
     </row>
     <row r="8" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="218" t="s">
+      <c r="A8" s="229" t="s">
         <v>221</v>
       </c>
-      <c r="B8" s="220" t="s">
+      <c r="B8" s="230" t="s">
         <v>222</v>
       </c>
-      <c r="C8" s="218" t="s">
+      <c r="C8" s="229" t="s">
         <v>223</v>
       </c>
       <c r="D8" s="176" t="s">
         <v>224</v>
       </c>
-      <c r="E8" s="221" t="s">
+      <c r="E8" s="231" t="s">
         <v>225</v>
       </c>
-      <c r="F8" s="224" t="s">
+      <c r="F8" s="225" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="224" t="s">
+      <c r="G8" s="225" t="s">
         <v>226</v>
       </c>
-      <c r="H8" s="224" t="s">
+      <c r="H8" s="225" t="s">
         <v>183</v>
       </c>
-      <c r="I8" s="222" t="s">
+      <c r="I8" s="232" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="222" t="s">
+      <c r="J8" s="232" t="s">
         <v>32</v>
       </c>
       <c r="K8" s="103"/>
-      <c r="L8" s="222"/>
-      <c r="M8" s="222"/>
+      <c r="L8" s="232"/>
+      <c r="M8" s="232"/>
       <c r="O8" s="27" t="s">
         <v>321</v>
       </c>
@@ -19258,75 +19321,75 @@
       <c r="V8" s="87"/>
     </row>
     <row r="9" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="219"/>
-      <c r="B9" s="219"/>
-      <c r="C9" s="219"/>
+      <c r="A9" s="221"/>
+      <c r="B9" s="221"/>
+      <c r="C9" s="221"/>
       <c r="D9" s="177" t="s">
         <v>227</v>
       </c>
-      <c r="E9" s="219"/>
-      <c r="F9" s="223"/>
-      <c r="G9" s="223"/>
-      <c r="H9" s="223"/>
-      <c r="I9" s="223"/>
-      <c r="J9" s="223"/>
+      <c r="E9" s="221"/>
+      <c r="F9" s="219"/>
+      <c r="G9" s="219"/>
+      <c r="H9" s="219"/>
+      <c r="I9" s="219"/>
+      <c r="J9" s="219"/>
       <c r="K9" s="103"/>
-      <c r="L9" s="223"/>
-      <c r="M9" s="223"/>
+      <c r="L9" s="219"/>
+      <c r="M9" s="219"/>
       <c r="S9" s="69"/>
     </row>
     <row r="10" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="219"/>
-      <c r="B10" s="219"/>
-      <c r="C10" s="219"/>
+      <c r="A10" s="221"/>
+      <c r="B10" s="221"/>
+      <c r="C10" s="221"/>
       <c r="D10" s="177" t="s">
         <v>228</v>
       </c>
-      <c r="E10" s="219"/>
-      <c r="F10" s="223"/>
-      <c r="G10" s="223"/>
-      <c r="H10" s="223"/>
-      <c r="I10" s="223"/>
-      <c r="J10" s="223"/>
+      <c r="E10" s="221"/>
+      <c r="F10" s="219"/>
+      <c r="G10" s="219"/>
+      <c r="H10" s="219"/>
+      <c r="I10" s="219"/>
+      <c r="J10" s="219"/>
       <c r="K10" s="103"/>
-      <c r="L10" s="223"/>
-      <c r="M10" s="223"/>
+      <c r="L10" s="219"/>
+      <c r="M10" s="219"/>
       <c r="S10" s="69"/>
     </row>
     <row r="11" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="219"/>
-      <c r="B11" s="219"/>
-      <c r="C11" s="219"/>
+      <c r="A11" s="221"/>
+      <c r="B11" s="221"/>
+      <c r="C11" s="221"/>
       <c r="D11" s="117" t="s">
         <v>229</v>
       </c>
-      <c r="E11" s="219"/>
-      <c r="F11" s="223"/>
-      <c r="G11" s="223"/>
-      <c r="H11" s="223"/>
-      <c r="I11" s="223"/>
-      <c r="J11" s="223"/>
+      <c r="E11" s="221"/>
+      <c r="F11" s="219"/>
+      <c r="G11" s="219"/>
+      <c r="H11" s="219"/>
+      <c r="I11" s="219"/>
+      <c r="J11" s="219"/>
       <c r="K11" s="118"/>
-      <c r="L11" s="223"/>
-      <c r="M11" s="223"/>
+      <c r="L11" s="219"/>
+      <c r="M11" s="219"/>
       <c r="S11" s="69"/>
     </row>
     <row r="12" spans="1:22" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="219"/>
-      <c r="B12" s="219"/>
-      <c r="C12" s="219"/>
+      <c r="A12" s="221"/>
+      <c r="B12" s="221"/>
+      <c r="C12" s="221"/>
       <c r="D12" s="117" t="s">
         <v>230</v>
       </c>
-      <c r="E12" s="219"/>
-      <c r="F12" s="223"/>
-      <c r="G12" s="223"/>
-      <c r="H12" s="223"/>
-      <c r="I12" s="223"/>
-      <c r="J12" s="223"/>
+      <c r="E12" s="221"/>
+      <c r="F12" s="219"/>
+      <c r="G12" s="219"/>
+      <c r="H12" s="219"/>
+      <c r="I12" s="219"/>
+      <c r="J12" s="219"/>
       <c r="K12" s="103"/>
-      <c r="L12" s="223"/>
-      <c r="M12" s="223"/>
+      <c r="L12" s="219"/>
+      <c r="M12" s="219"/>
       <c r="S12" s="69"/>
     </row>
     <row r="13" spans="1:22" ht="48" customHeight="1" x14ac:dyDescent="0.2">
@@ -19921,85 +19984,85 @@
     <mergeCell ref="H8:H12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
-    <cfRule type="cellIs" dxfId="309" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="313" priority="20" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F13:F24">
-    <cfRule type="cellIs" dxfId="308" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="312" priority="30" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="307" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="311" priority="33" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="306" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="310" priority="34" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="305" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="309" priority="35" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="304" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="308" priority="36" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H8 H13:H24">
-    <cfRule type="cellIs" dxfId="303" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="307" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="302" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="306" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F8">
-    <cfRule type="cellIs" dxfId="301" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="305" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="300" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="304" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="299" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="303" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="298" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="302" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J8 J13:J24">
-    <cfRule type="containsText" dxfId="297" priority="17" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="301" priority="17" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="296" priority="18" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="300" priority="18" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="295" priority="19" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="299" priority="19" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="294" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="298" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="293" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="297" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="292" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="296" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="291" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="295" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:S1">
-    <cfRule type="cellIs" dxfId="290" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="294" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="289" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="293" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="288" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="292" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="287" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="291" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20873,40 +20936,40 @@
       <c r="X16" s="87"/>
     </row>
     <row r="17" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="226" t="s">
+      <c r="A17" s="220" t="s">
         <v>221</v>
       </c>
-      <c r="B17" s="230" t="s">
+      <c r="B17" s="226" t="s">
         <v>222</v>
       </c>
-      <c r="C17" s="226" t="s">
+      <c r="C17" s="220" t="s">
         <v>223</v>
       </c>
       <c r="D17" s="178" t="s">
         <v>224</v>
       </c>
-      <c r="E17" s="227" t="s">
+      <c r="E17" s="222" t="s">
         <v>365</v>
       </c>
-      <c r="F17" s="224" t="s">
+      <c r="F17" s="225" t="s">
         <v>53</v>
       </c>
-      <c r="G17" s="231" t="s">
+      <c r="G17" s="227" t="s">
         <v>226</v>
       </c>
-      <c r="H17" s="231" t="s">
+      <c r="H17" s="227" t="s">
         <v>183</v>
       </c>
-      <c r="I17" s="225" t="s">
+      <c r="I17" s="218" t="s">
         <v>31</v>
       </c>
-      <c r="J17" s="225" t="s">
+      <c r="J17" s="218" t="s">
         <v>32</v>
       </c>
-      <c r="K17" s="232"/>
-      <c r="L17" s="225"/>
-      <c r="M17" s="229"/>
-      <c r="N17" s="229"/>
+      <c r="K17" s="228"/>
+      <c r="L17" s="218"/>
+      <c r="M17" s="224"/>
+      <c r="N17" s="224"/>
       <c r="P17" s="69" t="s">
         <v>321</v>
       </c>
@@ -20918,76 +20981,76 @@
       <c r="X17" s="91"/>
     </row>
     <row r="18" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="219"/>
-      <c r="B18" s="219"/>
-      <c r="C18" s="219"/>
+      <c r="A18" s="221"/>
+      <c r="B18" s="221"/>
+      <c r="C18" s="221"/>
       <c r="D18" s="179" t="s">
         <v>227</v>
       </c>
-      <c r="E18" s="228"/>
-      <c r="F18" s="223"/>
-      <c r="G18" s="223"/>
-      <c r="H18" s="223"/>
-      <c r="I18" s="223"/>
-      <c r="J18" s="223"/>
-      <c r="K18" s="223"/>
-      <c r="L18" s="223"/>
-      <c r="M18" s="223"/>
-      <c r="N18" s="223"/>
+      <c r="E18" s="223"/>
+      <c r="F18" s="219"/>
+      <c r="G18" s="219"/>
+      <c r="H18" s="219"/>
+      <c r="I18" s="219"/>
+      <c r="J18" s="219"/>
+      <c r="K18" s="219"/>
+      <c r="L18" s="219"/>
+      <c r="M18" s="219"/>
+      <c r="N18" s="219"/>
     </row>
     <row r="19" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="219"/>
-      <c r="B19" s="219"/>
-      <c r="C19" s="219"/>
+      <c r="A19" s="221"/>
+      <c r="B19" s="221"/>
+      <c r="C19" s="221"/>
       <c r="D19" s="179" t="s">
         <v>228</v>
       </c>
-      <c r="E19" s="228"/>
-      <c r="F19" s="223"/>
-      <c r="G19" s="223"/>
-      <c r="H19" s="223"/>
-      <c r="I19" s="223"/>
-      <c r="J19" s="223"/>
-      <c r="K19" s="223"/>
-      <c r="L19" s="223"/>
-      <c r="M19" s="223"/>
-      <c r="N19" s="223"/>
+      <c r="E19" s="223"/>
+      <c r="F19" s="219"/>
+      <c r="G19" s="219"/>
+      <c r="H19" s="219"/>
+      <c r="I19" s="219"/>
+      <c r="J19" s="219"/>
+      <c r="K19" s="219"/>
+      <c r="L19" s="219"/>
+      <c r="M19" s="219"/>
+      <c r="N19" s="219"/>
     </row>
     <row r="20" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="219"/>
-      <c r="B20" s="219"/>
-      <c r="C20" s="219"/>
+      <c r="A20" s="221"/>
+      <c r="B20" s="221"/>
+      <c r="C20" s="221"/>
       <c r="D20" s="105" t="s">
         <v>229</v>
       </c>
-      <c r="E20" s="228"/>
-      <c r="F20" s="223"/>
-      <c r="G20" s="223"/>
-      <c r="H20" s="223"/>
-      <c r="I20" s="223"/>
-      <c r="J20" s="223"/>
-      <c r="K20" s="223"/>
-      <c r="L20" s="223"/>
-      <c r="M20" s="223"/>
-      <c r="N20" s="223"/>
+      <c r="E20" s="223"/>
+      <c r="F20" s="219"/>
+      <c r="G20" s="219"/>
+      <c r="H20" s="219"/>
+      <c r="I20" s="219"/>
+      <c r="J20" s="219"/>
+      <c r="K20" s="219"/>
+      <c r="L20" s="219"/>
+      <c r="M20" s="219"/>
+      <c r="N20" s="219"/>
     </row>
     <row r="21" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="219"/>
-      <c r="B21" s="219"/>
-      <c r="C21" s="219"/>
+      <c r="A21" s="221"/>
+      <c r="B21" s="221"/>
+      <c r="C21" s="221"/>
       <c r="D21" s="105" t="s">
         <v>230</v>
       </c>
-      <c r="E21" s="228"/>
-      <c r="F21" s="223"/>
-      <c r="G21" s="223"/>
-      <c r="H21" s="223"/>
-      <c r="I21" s="223"/>
-      <c r="J21" s="223"/>
-      <c r="K21" s="223"/>
-      <c r="L21" s="223"/>
-      <c r="M21" s="223"/>
-      <c r="N21" s="223"/>
+      <c r="E21" s="223"/>
+      <c r="F21" s="219"/>
+      <c r="G21" s="219"/>
+      <c r="H21" s="219"/>
+      <c r="I21" s="219"/>
+      <c r="J21" s="219"/>
+      <c r="K21" s="219"/>
+      <c r="L21" s="219"/>
+      <c r="M21" s="219"/>
+      <c r="N21" s="219"/>
     </row>
     <row r="22" spans="1:24" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="87" t="s">
@@ -22977,68 +23040,68 @@
     <mergeCell ref="I17:I21"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F17 F22:F61">
-    <cfRule type="cellIs" dxfId="286" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="290" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H17 H22:H61">
-    <cfRule type="cellIs" dxfId="285" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="289" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="284" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="288" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F17 F22:F61">
-    <cfRule type="cellIs" dxfId="283" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="287" priority="23" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="282" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="286" priority="24" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="281" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="285" priority="25" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="280" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="284" priority="26" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J17 J22:J61">
-    <cfRule type="containsText" dxfId="279" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="283" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="278" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="282" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="277" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="281" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="276" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="280" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="275" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="279" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="274" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="278" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="273" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="277" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1:U1">
-    <cfRule type="cellIs" dxfId="272" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="276" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="271" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="275" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="270" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="274" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="269" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="273" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24353,54 +24416,54 @@
   </sheetData>
   <autoFilter ref="A1:J9" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <conditionalFormatting sqref="F2:F55">
-    <cfRule type="cellIs" dxfId="268" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="272" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H55">
-    <cfRule type="cellIs" dxfId="267" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="271" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="266" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="270" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F55">
-    <cfRule type="cellIs" dxfId="265" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="269" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="264" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="268" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="263" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="267" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="262" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="266" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J55">
-    <cfRule type="containsText" dxfId="261" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="265" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="260" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="264" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="259" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="263" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W1:AB1">
-    <cfRule type="cellIs" dxfId="258" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="262" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="257" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="261" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="256" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="260" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="255" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="259" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25530,54 +25593,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="254" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="258" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="253" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="257" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="252" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="256" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="251" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="255" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="250" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="254" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="249" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="253" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="248" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="252" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="247" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="251" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="246" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="250" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="245" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="249" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1:W1">
-    <cfRule type="cellIs" dxfId="244" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="248" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="243" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="247" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="242" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="246" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="241" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="245" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix(excel): apply 12 remaining text corrections on testing
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -133,7 +133,7 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Technical variable name required to match a column header in the CSV file (synthetic, anonymized representation of the real data), can appear in multiple languages.</t>
+    <t>A technical variable name is required to match a column header in the CSV file (a synthetic, anonymised representation of the real data).</t>
   </si>
   <si>
     <t>Mandatory</t>
@@ -209,7 +209,8 @@
     <t>csvw:propertyUrl</t>
   </si>
   <si>
-    <t>The propertyUrl may point to standard, controlled vocabularies, or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
+    <t>The propertyUrl may point to standard vocabularies, controlled vocabularies or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country
+For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
   </si>
   <si>
     <t>Recommended</t>
@@ -626,7 +627,7 @@
     <t>DCAT-AP v3</t>
   </si>
   <si>
-    <t>If applicable, add URI to connected dcat:Catalog</t>
+    <t>If applicable, enter the URI of the connected dcat:Catalog.</t>
   </si>
   <si>
     <t>hrishapes:CatalogShape</t>
@@ -698,7 +699,7 @@
     <t>Each catalogue contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
   </si>
   <si>
-    <t>Add URI to all datasets contained in this catalogue</t>
+    <t>Enter the URI for all datasets contained in this catalogue.</t>
   </si>
   <si>
     <t>hrishapes:DatasetShape</t>
@@ -811,7 +812,7 @@
     <t>https://definities.geostandaarden.nl/dcat-ap-nl/nl/</t>
   </si>
   <si>
-    <t>The licence under which the catalogue (with resource description) is made available.
+    <t>The licence under which the catalogue (with its resource description) is made available.
 The licences for Distributions and Data Services are not specified here. They are specified in the licence properties of their respective classes.</t>
   </si>
   <si>
@@ -899,7 +900,7 @@
     <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalogue and the Data Service via this property. While crucial for interoperability, this property is not relevant for end users to collect.</t>
   </si>
   <si>
-    <t>If applicable, add URI to dcat:DataService</t>
+    <t>If applicable, enter the URI for dcat:DataService.</t>
   </si>
   <si>
     <t>hrishapes:DataServiceShape</t>
@@ -965,7 +966,7 @@
     <t>http://publications.europa.eu/resource/authority/access-right</t>
   </si>
   <si>
-    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. It is foreseen that one of the three options has to be used: public, restricted, non-public.
+    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. One of the three options must be used: public, restricted, non-public.
     Open Data (Public): The dataset is available under general open data rules, such as those covered by the High Value Datasets Implementing Regulation.
     Protected Data (Restricted): The dataset contains protected data and is accessible only under specific conditions, as outlined in regulations like the Data Governance Act.
     Sensitive Data (Non-public): The dataset includes resources that may contain sensitive or personal information, falling under regulations such as the EHDS Regulation.
@@ -996,7 +997,7 @@
     <t>healthdcatap:analytics</t>
   </si>
   <si>
-    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would not be Distributions but rather DatasetServices.</t>
+    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would be Data Services rather than Distributions.</t>
   </si>
   <si>
     <t>custom:analytics</t>
@@ -1186,7 +1187,7 @@
     <t>custom:has_version</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Dataset that is another version of current Dataset</t>
+    <t>Enter the URI for the dcat:Dataset that is another version of the current Dataset.</t>
   </si>
   <si>
     <t>health condition of interest</t>
@@ -1512,8 +1513,8 @@
   <si>
     <t>This property makes use of another small class (prov:Attribution). There, you can choose one of the roles as listed in the controlled vocabulary and link that to a specific Agent (expressed with foaf:Agent).
 Repeat this property if you wish to specify multiple roles for the same agent.
-Refer to the Attribution class for more information how to fill this.
-Use this property if you would like to indicate the funder of the (research project that resulted in creation of the) dataset.
+Refer to the Attribution class for more information on how to fill this in.
+Use this property if you would like to indicate the funder of the dataset (or of the research project that resulted in its creation).
 The value for role in the Attribution class then becomes: https://standards.iso.org/iso/19115/resources/Codelists/gml/CI_RoleCode.xml#funder</t>
   </si>
   <si>
@@ -1882,7 +1883,7 @@
   </si>
   <si>
     <t>Note: This property will be deprecated in the next major release.
-Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use the following URL: http://purl.org/adms/publishertype/[type].</t>
+Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use URLs of the following form: http://purl.org/adms/publishertype/[type].</t>
   </si>
   <si>
     <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0).</t>
@@ -2131,7 +2132,7 @@
     <t>resource:format</t>
   </si>
   <si>
-    <t>Indicates the natural language used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
+    <t>Indicates the natural language used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions necessarily have a language; for example, those containing imaging data may not.
 Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
   </si>
   <si>

</xml_diff>

<commit_message>
fix(excel): apply 12 remaining text corrections on testing (#284)
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -133,7 +133,7 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Technical variable name required to match a column header in the CSV file (synthetic, anonymized representation of the real data), can appear in multiple languages.</t>
+    <t>A technical variable name is required to match a column header in the CSV file (a synthetic, anonymised representation of the real data).</t>
   </si>
   <si>
     <t>Mandatory</t>
@@ -209,7 +209,8 @@
     <t>csvw:propertyUrl</t>
   </si>
   <si>
-    <t>The propertyUrl may point to standard, controlled vocabularies, or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
+    <t>The propertyUrl may point to standard vocabularies, controlled vocabularies or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country
+For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
   </si>
   <si>
     <t>Recommended</t>
@@ -626,7 +627,7 @@
     <t>DCAT-AP v3</t>
   </si>
   <si>
-    <t>If applicable, add URI to connected dcat:Catalog</t>
+    <t>If applicable, enter the URI of the connected dcat:Catalog.</t>
   </si>
   <si>
     <t>hrishapes:CatalogShape</t>
@@ -698,7 +699,7 @@
     <t>Each catalogue contains one or more datasets. This property serves to link datasets to a catalogue. Therefore, a dataset is always contained inside a catalogue.</t>
   </si>
   <si>
-    <t>Add URI to all datasets contained in this catalogue</t>
+    <t>Enter the URI for all datasets contained in this catalogue.</t>
   </si>
   <si>
     <t>hrishapes:DatasetShape</t>
@@ -811,7 +812,7 @@
     <t>https://definities.geostandaarden.nl/dcat-ap-nl/nl/</t>
   </si>
   <si>
-    <t>The licence under which the catalogue (with resource description) is made available.
+    <t>The licence under which the catalogue (with its resource description) is made available.
 The licences for Distributions and Data Services are not specified here. They are specified in the licence properties of their respective classes.</t>
   </si>
   <si>
@@ -899,7 +900,7 @@
     <t>Some datasets may have real-time Data Services (e.g., Beacon API counting individuals). IT teams should define the relationship between the catalogue and the Data Service via this property. While crucial for interoperability, this property is not relevant for end users to collect.</t>
   </si>
   <si>
-    <t>If applicable, add URI to dcat:DataService</t>
+    <t>If applicable, enter the URI for dcat:DataService.</t>
   </si>
   <si>
     <t>hrishapes:DataServiceShape</t>
@@ -965,7 +966,7 @@
     <t>http://publications.europa.eu/resource/authority/access-right</t>
   </si>
   <si>
-    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. It is foreseen that one of the three options has to be used: public, restricted, non-public.
+    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. One of the three options must be used: public, restricted, non-public.
     Open Data (Public): The dataset is available under general open data rules, such as those covered by the High Value Datasets Implementing Regulation.
     Protected Data (Restricted): The dataset contains protected data and is accessible only under specific conditions, as outlined in regulations like the Data Governance Act.
     Sensitive Data (Non-public): The dataset includes resources that may contain sensitive or personal information, falling under regulations such as the EHDS Regulation.
@@ -996,7 +997,7 @@
     <t>healthdcatap:analytics</t>
   </si>
   <si>
-    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would not be Distributions but rather DatasetServices.</t>
+    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would be Data Services rather than Distributions.</t>
   </si>
   <si>
     <t>custom:analytics</t>
@@ -1186,7 +1187,7 @@
     <t>custom:has_version</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Dataset that is another version of current Dataset</t>
+    <t>Enter the URI for the dcat:Dataset that is another version of the current Dataset.</t>
   </si>
   <si>
     <t>health condition of interest</t>
@@ -1512,8 +1513,8 @@
   <si>
     <t>This property makes use of another small class (prov:Attribution). There, you can choose one of the roles as listed in the controlled vocabulary and link that to a specific Agent (expressed with foaf:Agent).
 Repeat this property if you wish to specify multiple roles for the same agent.
-Refer to the Attribution class for more information how to fill this.
-Use this property if you would like to indicate the funder of the (research project that resulted in creation of the) dataset.
+Refer to the Attribution class for more information on how to fill this in.
+Use this property if you would like to indicate the funder of the dataset (or of the research project that resulted in its creation).
 The value for role in the Attribution class then becomes: https://standards.iso.org/iso/19115/resources/Codelists/gml/CI_RoleCode.xml#funder</t>
   </si>
   <si>
@@ -1882,7 +1883,7 @@
   </si>
   <si>
     <t>Note: This property will be deprecated in the next major release.
-Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use the following URL: http://purl.org/adms/publishertype/[type].</t>
+Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use URLs of the following form: http://purl.org/adms/publishertype/[type].</t>
   </si>
   <si>
     <t>This property should be filled using ADMS vocabulary (http://purl.org/adms/publishertype/1.0).</t>
@@ -2131,7 +2132,7 @@
     <t>resource:format</t>
   </si>
   <si>
-    <t>Indicates the natural language used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
+    <t>Indicates the natural language used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions necessarily have a language; for example, those containing imaging data may not.
 Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
   </si>
   <si>

</xml_diff>

<commit_message>
fix: change requrement level for provenance statement label to mandatory
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0.xlsx
+++ b/Documents/Health-RI_v2.1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Library/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6BC147-5817-E84D-92E3-F4AFD43450AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB7EBB9-189E-AB42-ABC2-E936CFBA35A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="-19160" windowWidth="30240" windowHeight="17260" firstSheet="10" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="720" yWindow="-19160" windowWidth="30240" windowHeight="17260" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -3855,7 +3855,37 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="322">
+  <dxfs count="318">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -3868,6 +3898,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3898,6 +3958,36 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -3908,6 +3998,146 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -3918,6 +4148,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4058,6 +4298,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4068,6 +4328,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -4078,6 +4368,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4088,6 +4398,36 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4102,6 +4442,16 @@
       </font>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
@@ -4138,6 +4488,36 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4148,6 +4528,96 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -4158,6 +4628,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4252,7 +4732,17 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4268,6 +4758,46 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4292,7 +4822,37 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="2"/>
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4342,6 +4902,16 @@
       </font>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="4" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
@@ -4378,6 +4948,26 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -4388,6 +4978,246 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -4398,6 +5228,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="1"/>
       </font>
       <fill>
@@ -4492,7 +5332,67 @@
       </font>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.59999389629810485"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4503,946 +5403,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -9050,54 +9010,54 @@
   </sheetData>
   <autoFilter ref="A1:J24" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <conditionalFormatting sqref="F2:F54">
-    <cfRule type="cellIs" dxfId="240" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="236" priority="20" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H54">
-    <cfRule type="cellIs" dxfId="239" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="235" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="238" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="234" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F54">
-    <cfRule type="cellIs" dxfId="237" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="233" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="236" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="232" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="235" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="231" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="234" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="230" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J54">
-    <cfRule type="containsText" dxfId="233" priority="17" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="229" priority="17" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="232" priority="18" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="228" priority="18" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="231" priority="19" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="227" priority="19" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:T1">
-    <cfRule type="cellIs" dxfId="230" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="226" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="229" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="225" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="228" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="224" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="227" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="223" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9908,65 +9868,65 @@
     <mergeCell ref="G6:G10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="226" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="222" priority="11" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H6 H11 G12:I12">
-    <cfRule type="cellIs" dxfId="225" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="221" priority="12" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="224" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="220" priority="13" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F6 F11:F15">
-    <cfRule type="cellIs" dxfId="223" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="219" priority="14" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="222" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="218" priority="15" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="221" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="217" priority="16" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="220" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="216" priority="17" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J6">
-    <cfRule type="containsText" dxfId="219" priority="5" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="215" priority="5" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="218" priority="6" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="214" priority="6" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="217" priority="7" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="213" priority="7" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:J15">
-    <cfRule type="containsText" dxfId="216" priority="8" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="212" priority="8" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="215" priority="9" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="211" priority="9" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="214" priority="10" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="210" priority="10" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:R1">
-    <cfRule type="cellIs" dxfId="213" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="209" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="212" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="208" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="211" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="210" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="206" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11574,54 +11534,54 @@
   </sheetData>
   <autoFilter ref="A1:J23" xr:uid="{00000000-0009-0000-0000-00000B000000}"/>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="209" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="205" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="208" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="204" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="203" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="206" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="202" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="201" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="200" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="203" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="199" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="202" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="198" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="201" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="197" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="200" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="196" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:R1">
-    <cfRule type="cellIs" dxfId="199" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="195" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="194" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="197" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="193" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="192" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11840,49 +11800,49 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="195" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="191" priority="9" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="194" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="190" priority="10" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="193" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="11" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="188" priority="12" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="191" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="187" priority="13" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="190" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="186" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="185" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="184" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="187" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P1:U1">
-    <cfRule type="cellIs" dxfId="186" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="185" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="181" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="179" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12742,85 +12702,85 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A41:B42">
-    <cfRule type="cellIs" dxfId="182" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="179" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D40:E42">
-    <cfRule type="cellIs" dxfId="178" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="20" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="176" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="22" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F52">
-    <cfRule type="cellIs" dxfId="174" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="9" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="173" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="10" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="11" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="12" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="170" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="166" priority="13" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="169" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="165" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="24" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="167" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="163" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="164" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:X1">
-    <cfRule type="cellIs" dxfId="163" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="161" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="157" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="160" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12959,7 +12919,7 @@
         <v>787</v>
       </c>
       <c r="F2" s="33" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="G2" s="168" t="s">
         <v>29</v>
@@ -13258,89 +13218,89 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D11:E13">
-    <cfRule type="cellIs" dxfId="159" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="158" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="154" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="153" priority="21" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="152" priority="20" operator="equal">
       <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="21" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="22" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" dxfId="155" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="148" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F23 A12:B13">
-    <cfRule type="cellIs" dxfId="150" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="146" priority="15" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="149" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="145" priority="16" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="148" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="144" priority="17" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="18" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F23">
-    <cfRule type="cellIs" dxfId="146" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="142" priority="10" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2">
-    <cfRule type="cellIs" dxfId="145" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="141" priority="11" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="12" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="139" priority="13" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="14" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H12 H21:H23">
-    <cfRule type="cellIs" dxfId="141" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="137" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="24" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="139" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="135" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="134" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="1" operator="equal">
       <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -13564,35 +13524,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="135" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="134" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="130" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="129" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="128" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="130" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="123" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13795,35 +13755,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="126" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="125" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="120" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="118" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="121" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="115" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="114" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14026,35 +13986,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F3">
-    <cfRule type="cellIs" dxfId="117" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="5" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="cellIs" dxfId="116" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="6" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="7" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="8" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="9" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F3">
-    <cfRule type="cellIs" dxfId="112" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15098,14 +15058,14 @@
     <cfRule type="cellIs" dxfId="91" priority="25" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="26" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="90" priority="28" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="89" priority="27" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="28" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="88" priority="26" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
@@ -15145,25 +15105,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="77" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="77" priority="30" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="29" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="30" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F52">
-    <cfRule type="cellIs" dxfId="75" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="1" operator="equal">
       <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -15993,14 +15953,14 @@
     <cfRule type="cellIs" dxfId="71" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="20" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="70" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="69" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="22" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="68" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2">
@@ -16056,25 +16016,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H8 H10:H14 H16:H24 H26:H40 H49:H51">
-    <cfRule type="cellIs" dxfId="53" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="24" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="50" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="1" operator="equal">
       <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -16973,14 +16933,14 @@
     <cfRule type="cellIs" dxfId="47" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="20" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="46" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="45" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="22" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="44" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
@@ -17034,25 +16994,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="29" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="24" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
       <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -17979,14 +17939,14 @@
     <cfRule type="cellIs" dxfId="23" priority="19" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
-      <formula>"Recommended"</formula>
+    <cfRule type="cellIs" dxfId="22" priority="22" operator="equal">
+      <formula>"Conditional"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
-      <formula>"Conditional"</formula>
+    <cfRule type="cellIs" dxfId="20" priority="20" operator="equal">
+      <formula>"Recommended"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E3">
@@ -18040,25 +18000,25 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H9 H11:H15 H17:H25 H27:H41 H50:H52">
-    <cfRule type="cellIs" dxfId="5" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="24" operator="equal">
+      <formula>"needs review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="23" operator="greaterThan">
       <formula>"reviewd"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="24" operator="equal">
-      <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"Conditional"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"Mandatory"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Recommended"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Optional"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
-      <formula>"Recommended"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>"Mandatory"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
-      <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
@@ -18707,44 +18667,44 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F1 H1:I1">
-    <cfRule type="cellIs" dxfId="321" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="317" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="320" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="316" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="319" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="315" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="318" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="314" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="317" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="313" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="316" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="312" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="315" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="311" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="314" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="310" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M1:Q1">
-    <cfRule type="cellIs" dxfId="313" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="309" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="312" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="308" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="311" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="307" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="310" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="306" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19862,85 +19822,85 @@
     <mergeCell ref="H8:H12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
-    <cfRule type="cellIs" dxfId="309" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="305" priority="20" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F13:F24">
-    <cfRule type="cellIs" dxfId="308" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="304" priority="30" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="307" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="303" priority="33" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="306" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="302" priority="34" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="305" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="301" priority="35" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="304" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="300" priority="36" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H8 H13:H24">
-    <cfRule type="cellIs" dxfId="303" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="299" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="302" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="298" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F8">
-    <cfRule type="cellIs" dxfId="301" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="297" priority="9" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="300" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="296" priority="10" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="299" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="295" priority="11" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="298" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="294" priority="12" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J8 J13:J24">
-    <cfRule type="containsText" dxfId="297" priority="17" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="293" priority="17" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="296" priority="18" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="292" priority="18" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="295" priority="19" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="291" priority="19" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="294" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="290" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="293" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="289" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="292" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="288" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="291" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="287" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:S1">
-    <cfRule type="cellIs" dxfId="290" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="286" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="289" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="285" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="288" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="284" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="287" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="283" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22918,68 +22878,68 @@
     <mergeCell ref="I17:I21"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F17 F22:F61">
-    <cfRule type="cellIs" dxfId="286" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="282" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H17 H22:H61">
-    <cfRule type="cellIs" dxfId="285" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="281" priority="21" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="284" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="280" priority="22" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F17 F22:F61">
-    <cfRule type="cellIs" dxfId="283" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="279" priority="23" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="282" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="278" priority="24" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="281" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="277" priority="25" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="280" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="276" priority="26" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J17 J22:J61">
-    <cfRule type="containsText" dxfId="279" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="275" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="278" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="274" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="277" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="273" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1">
-    <cfRule type="cellIs" dxfId="276" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="272" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="275" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="271" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="274" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="270" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="273" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="269" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O1:U1">
-    <cfRule type="cellIs" dxfId="272" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="268" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="271" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="267" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="270" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="266" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="269" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="265" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24294,54 +24254,54 @@
   </sheetData>
   <autoFilter ref="A1:J9" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <conditionalFormatting sqref="F2:F55">
-    <cfRule type="cellIs" dxfId="268" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="264" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H55">
-    <cfRule type="cellIs" dxfId="267" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="263" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="266" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="262" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F55">
-    <cfRule type="cellIs" dxfId="265" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="261" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="264" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="260" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="263" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="259" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="262" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="258" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J55">
-    <cfRule type="containsText" dxfId="261" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="257" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="260" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="256" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="259" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="255" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W1:AB1">
-    <cfRule type="cellIs" dxfId="258" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="254" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="257" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="253" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="256" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="252" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="255" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="251" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25471,54 +25431,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="cellIs" dxfId="254" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="250" priority="12" operator="equal">
       <formula>"Not added"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H53">
-    <cfRule type="cellIs" dxfId="253" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="249" priority="13" operator="greaterThan">
       <formula>"reviewd"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="252" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="248" priority="14" operator="equal">
       <formula>"needs review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:I1 F1:F53">
-    <cfRule type="cellIs" dxfId="251" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="247" priority="5" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="250" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="246" priority="6" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="249" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="245" priority="7" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="248" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="244" priority="8" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J53">
-    <cfRule type="containsText" dxfId="247" priority="9" operator="containsText" text="Health and NL">
+    <cfRule type="containsText" dxfId="243" priority="9" operator="containsText" text="Health and NL">
       <formula>NOT(ISERROR(SEARCH("Health and NL",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="246" priority="10" operator="containsText" text="HealthDCAT-AP">
+    <cfRule type="containsText" dxfId="242" priority="10" operator="containsText" text="HealthDCAT-AP">
       <formula>NOT(ISERROR(SEARCH("HealthDCAT-AP",J2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="245" priority="11" operator="containsText" text="DCAT-AP NL">
+    <cfRule type="containsText" dxfId="241" priority="11" operator="containsText" text="DCAT-AP NL">
       <formula>NOT(ISERROR(SEARCH("DCAT-AP NL",J2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R1:W1">
-    <cfRule type="cellIs" dxfId="244" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="240" priority="1" operator="equal">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="243" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="239" priority="2" operator="equal">
       <formula>"Recommended"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="242" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="238" priority="3" operator="equal">
       <formula>"Mandatory"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="241" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="237" priority="4" operator="equal">
       <formula>"Conditional"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>